<commit_message>
update matrix cfg: 1. excel version 2. ring demo 3. support multi-range
</commit_message>
<xml_diff>
--- a/excel/excel_demo/regbank_demo.xlsx
+++ b/excel/excel_demo/regbank_demo.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="114">
   <si>
     <t>Access_Type</t>
   </si>
@@ -163,9 +163,6 @@
   </si>
   <si>
     <t>Size (in KB)</t>
-  </si>
-  <si>
-    <t>APB3</t>
   </si>
   <si>
     <t>Interface Width</t>
@@ -999,7 +996,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="C4" s="16"/>
       <c r="D4" s="16"/>
@@ -1015,7 +1012,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B5" s="15">
         <v>16</v>
@@ -1053,10 +1050,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="18" t="s">
         <v>51</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>52</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
@@ -1102,51 +1099,51 @@
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" s="21" t="s">
         <v>53</v>
-      </c>
-      <c r="B10" s="21" t="s">
-        <v>54</v>
       </c>
       <c r="C10" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D10" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10" s="14" t="s">
         <v>55</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>56</v>
       </c>
       <c r="F10" s="14" t="s">
         <v>1</v>
       </c>
       <c r="G10" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="H10" s="14" t="s">
+      <c r="I10" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="I10" s="14" t="s">
+      <c r="J10" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="K10" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="J10" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="K10" s="14" t="s">
+      <c r="L10" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="L10" s="14" t="s">
+      <c r="M10" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="M10" s="14" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
+      <c r="A11" s="16" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="20.25">
-      <c r="A11" s="16" t="s">
+      <c r="B11" s="22" t="s">
         <v>63</v>
-      </c>
-      <c r="B11" s="22" t="s">
-        <v>64</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>9</v>
@@ -1158,23 +1155,23 @@
       <c r="H11" s="16"/>
       <c r="I11" s="16"/>
       <c r="J11" s="16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K11" s="16"/>
       <c r="L11" s="16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="M11" s="16"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="20.25">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="16"/>
       <c r="B12" s="4"/>
       <c r="C12" s="16"/>
       <c r="D12" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" s="16" t="s">
         <v>67</v>
-      </c>
-      <c r="E12" s="16" t="s">
-        <v>68</v>
       </c>
       <c r="F12" s="16" t="s">
         <v>6</v>
@@ -1186,24 +1183,24 @@
         <v>10</v>
       </c>
       <c r="I12" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="J12" s="16" t="s">
         <v>69</v>
-      </c>
-      <c r="J12" s="16" t="s">
-        <v>70</v>
       </c>
       <c r="K12" s="16"/>
       <c r="L12" s="16"/>
       <c r="M12" s="16"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="20.25">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="16"/>
       <c r="B13" s="4"/>
       <c r="C13" s="16"/>
       <c r="D13" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="E13" s="16" t="s">
         <v>71</v>
-      </c>
-      <c r="E13" s="16" t="s">
-        <v>72</v>
       </c>
       <c r="F13" s="16" t="s">
         <v>6</v>
@@ -1215,24 +1212,24 @@
         <v>10</v>
       </c>
       <c r="I13" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="J13" s="16" t="s">
         <v>73</v>
-      </c>
-      <c r="J13" s="16" t="s">
-        <v>74</v>
       </c>
       <c r="K13" s="16"/>
       <c r="L13" s="16"/>
       <c r="M13" s="16"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="20.25">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="16"/>
       <c r="B14" s="4"/>
       <c r="C14" s="16"/>
       <c r="D14" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="E14" s="16" t="s">
         <v>75</v>
-      </c>
-      <c r="E14" s="16" t="s">
-        <v>76</v>
       </c>
       <c r="F14" s="16" t="s">
         <v>6</v>
@@ -1244,24 +1241,24 @@
         <v>10</v>
       </c>
       <c r="I14" s="16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J14" s="16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="K14" s="16"/>
       <c r="L14" s="16"/>
       <c r="M14" s="16"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="20.25">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="16"/>
       <c r="B15" s="4"/>
       <c r="C15" s="16"/>
       <c r="D15" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="E15" s="16" t="s">
         <v>78</v>
-      </c>
-      <c r="E15" s="16" t="s">
-        <v>79</v>
       </c>
       <c r="F15" s="16" t="s">
         <v>6</v>
@@ -1273,21 +1270,21 @@
         <v>15</v>
       </c>
       <c r="I15" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="J15" s="16" t="s">
         <v>80</v>
-      </c>
-      <c r="J15" s="16" t="s">
-        <v>81</v>
       </c>
       <c r="K15" s="16"/>
       <c r="L15" s="16"/>
       <c r="M15" s="16"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="20.25">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="B16" s="22" t="s">
         <v>82</v>
-      </c>
-      <c r="B16" s="22" t="s">
-        <v>83</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>9</v>
@@ -1299,13 +1296,13 @@
       <c r="H16" s="16"/>
       <c r="I16" s="16"/>
       <c r="J16" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="K16" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="K16" s="9" t="s">
+      <c r="L16" s="9" t="s">
         <v>85</v>
-      </c>
-      <c r="L16" s="9" t="s">
-        <v>86</v>
       </c>
       <c r="M16" s="9"/>
     </row>
@@ -1314,10 +1311,10 @@
       <c r="B17" s="4"/>
       <c r="C17" s="16"/>
       <c r="D17" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="E17" s="16" t="s">
         <v>67</v>
-      </c>
-      <c r="E17" s="16" t="s">
-        <v>68</v>
       </c>
       <c r="F17" s="16" t="s">
         <v>6</v>
@@ -1329,13 +1326,13 @@
         <v>15</v>
       </c>
       <c r="I17" s="16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J17" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="K17" s="9" t="s">
         <v>87</v>
-      </c>
-      <c r="K17" s="9" t="s">
-        <v>88</v>
       </c>
       <c r="L17" s="9"/>
       <c r="M17" s="9"/>
@@ -1345,10 +1342,10 @@
       <c r="B18" s="4"/>
       <c r="C18" s="16"/>
       <c r="D18" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F18" s="16" t="s">
         <v>6</v>
@@ -1360,13 +1357,13 @@
         <v>15</v>
       </c>
       <c r="I18" s="16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J18" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="K18" s="9" t="s">
         <v>90</v>
-      </c>
-      <c r="K18" s="9" t="s">
-        <v>91</v>
       </c>
       <c r="L18" s="9"/>
       <c r="M18" s="9"/>
@@ -1376,10 +1373,10 @@
       <c r="B19" s="4"/>
       <c r="C19" s="16"/>
       <c r="D19" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="E19" s="16" t="s">
         <v>75</v>
-      </c>
-      <c r="E19" s="16" t="s">
-        <v>76</v>
       </c>
       <c r="F19" s="16" t="s">
         <v>6</v>
@@ -1391,10 +1388,10 @@
         <v>10</v>
       </c>
       <c r="I19" s="16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J19" s="16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="K19" s="9"/>
       <c r="L19" s="9"/>
@@ -1405,10 +1402,10 @@
       <c r="B20" s="4"/>
       <c r="C20" s="16"/>
       <c r="D20" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="E20" s="16" t="s">
         <v>78</v>
-      </c>
-      <c r="E20" s="16" t="s">
-        <v>79</v>
       </c>
       <c r="F20" s="16" t="s">
         <v>6</v>
@@ -1420,10 +1417,10 @@
         <v>15</v>
       </c>
       <c r="I20" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="J20" s="16" t="s">
         <v>80</v>
-      </c>
-      <c r="J20" s="16" t="s">
-        <v>81</v>
       </c>
       <c r="K20" s="16"/>
       <c r="L20" s="9"/>
@@ -1431,10 +1428,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="B21" s="22" t="s">
         <v>92</v>
-      </c>
-      <c r="B21" s="22" t="s">
-        <v>93</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>9</v>
@@ -1446,11 +1443,11 @@
       <c r="H21" s="16"/>
       <c r="I21" s="16"/>
       <c r="J21" s="16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="K21" s="9"/>
       <c r="L21" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M21" s="9"/>
     </row>
@@ -1459,10 +1456,10 @@
       <c r="B22" s="4"/>
       <c r="C22" s="16"/>
       <c r="D22" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="E22" s="16" t="s">
         <v>67</v>
-      </c>
-      <c r="E22" s="16" t="s">
-        <v>68</v>
       </c>
       <c r="F22" s="16" t="s">
         <v>6</v>
@@ -1474,10 +1471,10 @@
         <v>10</v>
       </c>
       <c r="I22" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="J22" s="16" t="s">
         <v>69</v>
-      </c>
-      <c r="J22" s="16" t="s">
-        <v>70</v>
       </c>
       <c r="K22" s="9"/>
       <c r="L22" s="9"/>
@@ -1488,10 +1485,10 @@
       <c r="B23" s="4"/>
       <c r="C23" s="16"/>
       <c r="D23" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="E23" s="16" t="s">
         <v>71</v>
-      </c>
-      <c r="E23" s="16" t="s">
-        <v>72</v>
       </c>
       <c r="F23" s="16" t="s">
         <v>6</v>
@@ -1503,10 +1500,10 @@
         <v>10</v>
       </c>
       <c r="I23" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="J23" s="16" t="s">
         <v>73</v>
-      </c>
-      <c r="J23" s="16" t="s">
-        <v>74</v>
       </c>
       <c r="K23" s="9"/>
       <c r="L23" s="9"/>
@@ -1517,10 +1514,10 @@
       <c r="B24" s="4"/>
       <c r="C24" s="16"/>
       <c r="D24" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="E24" s="16" t="s">
         <v>75</v>
-      </c>
-      <c r="E24" s="16" t="s">
-        <v>76</v>
       </c>
       <c r="F24" s="16" t="s">
         <v>6</v>
@@ -1532,10 +1529,10 @@
         <v>10</v>
       </c>
       <c r="I24" s="16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J24" s="16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="K24" s="9"/>
       <c r="L24" s="9"/>
@@ -1546,10 +1543,10 @@
       <c r="B25" s="4"/>
       <c r="C25" s="16"/>
       <c r="D25" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="E25" s="16" t="s">
         <v>78</v>
-      </c>
-      <c r="E25" s="16" t="s">
-        <v>79</v>
       </c>
       <c r="F25" s="16" t="s">
         <v>6</v>
@@ -1561,81 +1558,81 @@
         <v>15</v>
       </c>
       <c r="I25" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="J25" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="J25" s="16" t="s">
-        <v>81</v>
-      </c>
       <c r="K25" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5">
       <c r="A26" s="16" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B26" s="22" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>14</v>
       </c>
       <c r="D26" s="16"/>
       <c r="E26" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F26" s="16"/>
       <c r="G26" s="16"/>
       <c r="H26" s="16"/>
       <c r="I26" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="J26" s="16" t="s">
         <v>99</v>
-      </c>
-      <c r="J26" s="16" t="s">
-        <v>100</v>
       </c>
       <c r="K26" s="16"/>
       <c r="L26" s="16"/>
       <c r="M26" s="16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5">
       <c r="A27" s="16" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B27" s="22" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>14</v>
       </c>
       <c r="D27" s="16"/>
       <c r="E27" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F27" s="16"/>
       <c r="G27" s="16"/>
       <c r="H27" s="16"/>
       <c r="I27" s="16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J27" s="16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K27" s="16"/>
       <c r="L27" s="16"/>
       <c r="M27" s="16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5">
       <c r="A28" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="B28" s="22" t="s">
         <v>104</v>
-      </c>
-      <c r="B28" s="22" t="s">
-        <v>105</v>
       </c>
       <c r="C28" s="16" t="s">
         <v>16</v>
@@ -1647,7 +1644,7 @@
       <c r="H28" s="16"/>
       <c r="I28" s="16"/>
       <c r="J28" s="16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K28" s="16"/>
       <c r="L28" s="16"/>
@@ -1658,17 +1655,17 @@
       <c r="B29" s="22"/>
       <c r="C29" s="16"/>
       <c r="D29" s="16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E29" s="16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F29" s="16"/>
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
       <c r="I29" s="16"/>
       <c r="J29" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K29" s="16"/>
       <c r="L29" s="16"/>
@@ -1679,17 +1676,17 @@
       <c r="B30" s="22"/>
       <c r="C30" s="16"/>
       <c r="D30" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="E30" s="16" t="s">
         <v>109</v>
-      </c>
-      <c r="E30" s="16" t="s">
-        <v>110</v>
       </c>
       <c r="F30" s="16"/>
       <c r="G30" s="16"/>
       <c r="H30" s="16"/>
       <c r="I30" s="16"/>
       <c r="J30" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K30" s="16"/>
       <c r="L30" s="16"/>
@@ -1697,10 +1694,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="19.5">
       <c r="A31" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="B31" s="22" t="s">
         <v>112</v>
-      </c>
-      <c r="B31" s="22" t="s">
-        <v>113</v>
       </c>
       <c r="C31" s="16" t="s">
         <v>16</v>
@@ -1712,7 +1709,7 @@
       <c r="H31" s="16"/>
       <c r="I31" s="16"/>
       <c r="J31" s="16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K31" s="16"/>
       <c r="L31" s="16"/>
@@ -1723,17 +1720,17 @@
       <c r="B32" s="22"/>
       <c r="C32" s="16"/>
       <c r="D32" s="16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E32" s="16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F32" s="16"/>
       <c r="G32" s="16"/>
       <c r="H32" s="16"/>
       <c r="I32" s="16"/>
       <c r="J32" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K32" s="16"/>
       <c r="L32" s="16"/>
@@ -1744,17 +1741,17 @@
       <c r="B33" s="22"/>
       <c r="C33" s="16"/>
       <c r="D33" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E33" s="16" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F33" s="16"/>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
       <c r="I33" s="16"/>
       <c r="J33" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K33" s="16"/>
       <c r="L33" s="16"/>

</xml_diff>